<commit_message>
fix: mit black formatiert
</commit_message>
<xml_diff>
--- a/docs/protocols/DailyScrum_01.09.xlsx
+++ b/docs/protocols/DailyScrum_01.09.xlsx
@@ -398,6 +398,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J13"/>
+  <cols>
+    <col min="2" max="2" width="10.16796875" customWidth="1"/>
+    <col min="3" max="3" width="11.8359375" customWidth="1"/>
+    <col min="4" max="4" width="13.61328125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>